<commit_message>
create account script and bulk uploads script completed ready for testing
</commit_message>
<xml_diff>
--- a/account_employee_setup/positive_imports/employee_basic.xlsx
+++ b/account_employee_setup/positive_imports/employee_basic.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henrycole/Desktop/account_employee_setup/positive_imports/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/henrycole/Desktop/automation/hr_regression/account_employee_setup/positive_imports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F47FA5-E570-EE49-BFA5-1087A0D22547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3F0D5F-C997-354B-A9CC-D0EC0796BAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30120" yWindow="4520" windowWidth="23520" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="employee_basic_template" sheetId="1" r:id="rId1"/>
@@ -71,19 +71,19 @@
     <t>02/01/2022</t>
   </si>
   <si>
-    <t>employee@hr_regression.com</t>
-  </si>
-  <si>
-    <t>line@hr_regression.com</t>
-  </si>
-  <si>
-    <t>finance@hr_regression.com</t>
-  </si>
-  <si>
-    <t>contractor@hr_regression.com</t>
-  </si>
-  <si>
-    <t>volunteer@hr_regression.com</t>
+    <t>employee@hr-regression.com</t>
+  </si>
+  <si>
+    <t>line@hr-regression.com</t>
+  </si>
+  <si>
+    <t>finance@hr-regression.com</t>
+  </si>
+  <si>
+    <t>contractor@hr-regression.com</t>
+  </si>
+  <si>
+    <t>volunteer@hr-regression.com</t>
   </si>
 </sst>
 </file>

</xml_diff>